<commit_message>
Rebuild candidates_final: novelty-prioritised (cap 1.5, wider bounds, UTS floor 520)
- Objective switched to discovery: find new distinct 7xxx alloys with good (not peak) strength
- 5 candidates at novelty 1.5, UTS 521-597 MPa, diverse chemistries
- README + xlsx + flow diagram updated to match; novelty_sweep.py added

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/candidates_final.xlsx
+++ b/data/candidates_final.xlsx
@@ -585,22 +585,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>87.63</v>
+        <v>87.27</v>
       </c>
       <c r="C2" t="n">
-        <v>7.48</v>
+        <v>6.92</v>
       </c>
       <c r="D2" t="n">
-        <v>2.61</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>1.52</v>
+        <v>2.22</v>
       </c>
       <c r="F2" t="n">
-        <v>0.34</v>
+        <v>0.24</v>
       </c>
       <c r="G2" t="n">
-        <v>0.17</v>
+        <v>0.09</v>
       </c>
       <c r="H2" t="n">
         <v>0.15</v>
@@ -609,34 +609,34 @@
         <v>0.1</v>
       </c>
       <c r="J2" t="n">
-        <v>488.48</v>
+        <v>494.6</v>
       </c>
       <c r="K2" t="n">
-        <v>104.11</v>
+        <v>127.01</v>
       </c>
       <c r="L2" t="n">
-        <v>24.24</v>
+        <v>44.32</v>
       </c>
       <c r="M2" t="n">
-        <v>634.85</v>
+        <v>597.13</v>
       </c>
       <c r="N2" t="n">
-        <v>13.6</v>
+        <v>24.88</v>
       </c>
       <c r="O2" t="n">
-        <v>554.9299999999999</v>
+        <v>535.67</v>
       </c>
       <c r="P2" t="n">
-        <v>25.02</v>
+        <v>25.84</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.03</v>
+        <v>10.57</v>
       </c>
       <c r="R2" t="n">
-        <v>1.13</v>
+        <v>1.5</v>
       </c>
       <c r="S2" t="n">
-        <v>621.2525024414062</v>
+        <v>572.2451</v>
       </c>
     </row>
     <row r="3">
@@ -644,22 +644,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>87.83</v>
+        <v>88.34</v>
       </c>
       <c r="C3" t="n">
-        <v>8.02</v>
+        <v>8.32</v>
       </c>
       <c r="D3" t="n">
-        <v>2.66</v>
+        <v>1.35</v>
       </c>
       <c r="E3" t="n">
-        <v>0.88</v>
+        <v>1.53</v>
       </c>
       <c r="F3" t="n">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="G3" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="H3" t="n">
         <v>0.15</v>
@@ -668,34 +668,34 @@
         <v>0.1</v>
       </c>
       <c r="J3" t="n">
-        <v>483.02</v>
+        <v>493.19</v>
       </c>
       <c r="K3" t="n">
-        <v>105.72</v>
+        <v>109.47</v>
       </c>
       <c r="L3" t="n">
-        <v>25.07</v>
+        <v>15.76</v>
       </c>
       <c r="M3" t="n">
-        <v>640.48</v>
+        <v>557.36</v>
       </c>
       <c r="N3" t="n">
-        <v>19.32</v>
+        <v>23.22</v>
       </c>
       <c r="O3" t="n">
-        <v>589.01</v>
+        <v>466.79</v>
       </c>
       <c r="P3" t="n">
-        <v>28.2</v>
+        <v>33.78</v>
       </c>
       <c r="Q3" t="n">
-        <v>11.08</v>
+        <v>16.55</v>
       </c>
       <c r="R3" t="n">
-        <v>1.24</v>
+        <v>1.5</v>
       </c>
       <c r="S3" t="n">
-        <v>621.1641845703125</v>
+        <v>534.1482</v>
       </c>
     </row>
     <row r="4">
@@ -703,22 +703,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>87.26000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="C4" t="n">
-        <v>7.11</v>
+        <v>5.48</v>
       </c>
       <c r="D4" t="n">
-        <v>2.56</v>
+        <v>2.47</v>
       </c>
       <c r="E4" t="n">
-        <v>2.25</v>
+        <v>0.51</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4</v>
+        <v>0.16</v>
       </c>
       <c r="G4" t="n">
-        <v>0.17</v>
+        <v>0.33</v>
       </c>
       <c r="H4" t="n">
         <v>0.15</v>
@@ -727,34 +727,34 @@
         <v>0.1</v>
       </c>
       <c r="J4" t="n">
-        <v>464</v>
+        <v>461.28</v>
       </c>
       <c r="K4" t="n">
-        <v>100.17</v>
+        <v>103.76</v>
       </c>
       <c r="L4" t="n">
-        <v>35.08</v>
+        <v>59.25</v>
       </c>
       <c r="M4" t="n">
-        <v>639.3099999999999</v>
+        <v>536.67</v>
       </c>
       <c r="N4" t="n">
-        <v>21.39</v>
+        <v>22.5</v>
       </c>
       <c r="O4" t="n">
-        <v>566.37</v>
+        <v>469.33</v>
       </c>
       <c r="P4" t="n">
-        <v>29.97</v>
+        <v>22.9</v>
       </c>
       <c r="Q4" t="n">
-        <v>11.15</v>
+        <v>10.29</v>
       </c>
       <c r="R4" t="n">
-        <v>1.11</v>
+        <v>1.5</v>
       </c>
       <c r="S4" t="n">
-        <v>617.9280395507812</v>
+        <v>514.16565</v>
       </c>
     </row>
     <row r="5">
@@ -762,22 +762,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>87.90000000000001</v>
+        <v>90.69</v>
       </c>
       <c r="C5" t="n">
-        <v>8.06</v>
+        <v>5.18</v>
       </c>
       <c r="D5" t="n">
-        <v>2.12</v>
+        <v>1.86</v>
       </c>
       <c r="E5" t="n">
-        <v>1.56</v>
+        <v>1.54</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01</v>
+        <v>0.41</v>
       </c>
       <c r="G5" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="H5" t="n">
         <v>0.15</v>
@@ -786,34 +786,34 @@
         <v>0.1</v>
       </c>
       <c r="J5" t="n">
-        <v>484.53</v>
+        <v>479.98</v>
       </c>
       <c r="K5" t="n">
-        <v>106.55</v>
+        <v>96.47</v>
       </c>
       <c r="L5" t="n">
-        <v>22.66</v>
+        <v>20.06</v>
       </c>
       <c r="M5" t="n">
-        <v>632.13</v>
+        <v>525.89</v>
       </c>
       <c r="N5" t="n">
-        <v>23.28</v>
+        <v>17.84</v>
       </c>
       <c r="O5" t="n">
-        <v>553.28</v>
+        <v>406.15</v>
       </c>
       <c r="P5" t="n">
-        <v>30.52</v>
+        <v>16.99</v>
       </c>
       <c r="Q5" t="n">
-        <v>16.22</v>
+        <v>14.37</v>
       </c>
       <c r="R5" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="S5" t="n">
-        <v>608.8536987304688</v>
+        <v>508.04645</v>
       </c>
     </row>
     <row r="6">
@@ -821,22 +821,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>87.92</v>
+        <v>88.89</v>
       </c>
       <c r="C6" t="n">
-        <v>6.52</v>
+        <v>5.95</v>
       </c>
       <c r="D6" t="n">
-        <v>2.54</v>
+        <v>3.13</v>
       </c>
       <c r="E6" t="n">
-        <v>2.23</v>
+        <v>1.75</v>
       </c>
       <c r="F6" t="n">
-        <v>0.39</v>
+        <v>0.03</v>
       </c>
       <c r="G6" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0.15</v>
@@ -845,34 +845,34 @@
         <v>0.1</v>
       </c>
       <c r="J6" t="n">
-        <v>486.42</v>
+        <v>463.26</v>
       </c>
       <c r="K6" t="n">
-        <v>109.97</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>33.93</v>
+        <v>19.65</v>
       </c>
       <c r="M6" t="n">
-        <v>619.49</v>
+        <v>520.77</v>
       </c>
       <c r="N6" t="n">
-        <v>12.61</v>
+        <v>37.51</v>
       </c>
       <c r="O6" t="n">
-        <v>527.55</v>
+        <v>425.33</v>
       </c>
       <c r="P6" t="n">
-        <v>19.6</v>
+        <v>34.99</v>
       </c>
       <c r="Q6" t="n">
-        <v>10.7</v>
+        <v>13.91</v>
       </c>
       <c r="R6" t="n">
-        <v>1.14</v>
+        <v>1.5</v>
       </c>
       <c r="S6" t="n">
-        <v>606.8843383789062</v>
+        <v>483.25238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>